<commit_message>
Lille : remplit DE/DV/EB (vides à cause du bug corrigé en beda83f)
87 lignes x 3 colonnes -- rattrape le run déjà commis avant le fix du
code.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/state/2275_lille.xlsx
+++ b/state/2275_lille.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" tabRatio="600" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuille" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="RUP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feuille" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RUP" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -1633,7 +1633,7 @@
       <c r="EK1" s="5" t="n"/>
       <c r="EL1" s="5" t="inlineStr">
         <is>
-          <t>                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                              </t>
+          <t xml:space="preserve">                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                                              </t>
         </is>
       </c>
       <c r="EM1" s="5" t="n"/>
@@ -4389,6 +4389,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF5" t="inlineStr">
         <is>
           <t>O</t>
@@ -4469,6 +4474,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW5" t="inlineStr">
         <is>
           <t>N</t>
@@ -4490,6 +4500,11 @@
         </is>
       </c>
       <c r="EA5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -5316,6 +5331,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF6" t="inlineStr">
         <is>
           <t>O</t>
@@ -5396,6 +5416,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW6" t="inlineStr">
         <is>
           <t>N</t>
@@ -5417,6 +5442,11 @@
         </is>
       </c>
       <c r="EA6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -6243,6 +6273,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF7" t="inlineStr">
         <is>
           <t>O</t>
@@ -6323,6 +6358,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW7" t="inlineStr">
         <is>
           <t>N</t>
@@ -6344,6 +6384,11 @@
         </is>
       </c>
       <c r="EA7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB7" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -7170,6 +7215,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF8" t="inlineStr">
         <is>
           <t>O</t>
@@ -7250,6 +7300,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW8" t="inlineStr">
         <is>
           <t>N</t>
@@ -7271,6 +7326,11 @@
         </is>
       </c>
       <c r="EA8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB8" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -8097,6 +8157,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF9" t="inlineStr">
         <is>
           <t>O</t>
@@ -8177,6 +8242,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW9" t="inlineStr">
         <is>
           <t>N</t>
@@ -8198,6 +8268,11 @@
         </is>
       </c>
       <c r="EA9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -9024,6 +9099,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF10" t="inlineStr">
         <is>
           <t>O</t>
@@ -9104,6 +9184,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW10" t="inlineStr">
         <is>
           <t>N</t>
@@ -9125,6 +9210,11 @@
         </is>
       </c>
       <c r="EA10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB10" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -9951,6 +10041,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF11" t="inlineStr">
         <is>
           <t>O</t>
@@ -10031,6 +10126,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW11" t="inlineStr">
         <is>
           <t>N</t>
@@ -10052,6 +10152,11 @@
         </is>
       </c>
       <c r="EA11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB11" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -10878,6 +10983,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF12" t="inlineStr">
         <is>
           <t>O</t>
@@ -10958,6 +11068,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW12" t="inlineStr">
         <is>
           <t>N</t>
@@ -10979,6 +11094,11 @@
         </is>
       </c>
       <c r="EA12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB12" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -11805,6 +11925,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF13" t="inlineStr">
         <is>
           <t>O</t>
@@ -11885,6 +12010,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW13" t="inlineStr">
         <is>
           <t>N</t>
@@ -11906,6 +12036,11 @@
         </is>
       </c>
       <c r="EA13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB13" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -12732,6 +12867,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF14" t="inlineStr">
         <is>
           <t>O</t>
@@ -12812,6 +12952,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW14" t="inlineStr">
         <is>
           <t>N</t>
@@ -12833,6 +12978,11 @@
         </is>
       </c>
       <c r="EA14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB14" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -13659,6 +13809,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF15" t="inlineStr">
         <is>
           <t>O</t>
@@ -13739,6 +13894,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW15" t="inlineStr">
         <is>
           <t>N</t>
@@ -13760,6 +13920,11 @@
         </is>
       </c>
       <c r="EA15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB15" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -14586,6 +14751,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF16" t="inlineStr">
         <is>
           <t>O</t>
@@ -14666,6 +14836,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW16" t="inlineStr">
         <is>
           <t>N</t>
@@ -14687,6 +14862,11 @@
         </is>
       </c>
       <c r="EA16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB16" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -15513,6 +15693,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF17" t="inlineStr">
         <is>
           <t>O</t>
@@ -15593,6 +15778,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW17" t="inlineStr">
         <is>
           <t>N</t>
@@ -15614,6 +15804,11 @@
         </is>
       </c>
       <c r="EA17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB17" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -16440,6 +16635,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF18" t="inlineStr">
         <is>
           <t>O</t>
@@ -16520,6 +16720,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW18" t="inlineStr">
         <is>
           <t>N</t>
@@ -16541,6 +16746,11 @@
         </is>
       </c>
       <c r="EA18" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB18" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -17367,6 +17577,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE19" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF19" t="inlineStr">
         <is>
           <t>O</t>
@@ -17447,6 +17662,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV19" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW19" t="inlineStr">
         <is>
           <t>N</t>
@@ -17468,6 +17688,11 @@
         </is>
       </c>
       <c r="EA19" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB19" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -18294,6 +18519,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF20" t="inlineStr">
         <is>
           <t>O</t>
@@ -18374,6 +18604,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW20" t="inlineStr">
         <is>
           <t>O</t>
@@ -18395,6 +18630,11 @@
         </is>
       </c>
       <c r="EA20" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB20" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -19221,6 +19461,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE21" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF21" t="inlineStr">
         <is>
           <t>O</t>
@@ -19301,6 +19546,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV21" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW21" t="inlineStr">
         <is>
           <t>O</t>
@@ -19322,6 +19572,11 @@
         </is>
       </c>
       <c r="EA21" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -20148,6 +20403,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF22" t="inlineStr">
         <is>
           <t>O</t>
@@ -20228,6 +20488,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW22" t="inlineStr">
         <is>
           <t>O</t>
@@ -20249,6 +20514,11 @@
         </is>
       </c>
       <c r="EA22" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB22" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -21075,6 +21345,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF23" t="inlineStr">
         <is>
           <t>O</t>
@@ -21155,6 +21430,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW23" t="inlineStr">
         <is>
           <t>O</t>
@@ -21176,6 +21456,11 @@
         </is>
       </c>
       <c r="EA23" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB23" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -22002,6 +22287,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF24" t="inlineStr">
         <is>
           <t>O</t>
@@ -22082,6 +22372,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW24" t="inlineStr">
         <is>
           <t>O</t>
@@ -22103,6 +22398,11 @@
         </is>
       </c>
       <c r="EA24" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB24" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -22919,6 +23219,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF25" t="inlineStr">
         <is>
           <t>O</t>
@@ -22999,6 +23304,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW25" t="inlineStr">
         <is>
           <t>O</t>
@@ -23020,6 +23330,11 @@
         </is>
       </c>
       <c r="EA25" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB25" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -23846,6 +24161,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE26" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF26" t="inlineStr">
         <is>
           <t>O</t>
@@ -23926,6 +24246,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV26" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW26" t="inlineStr">
         <is>
           <t>O</t>
@@ -23947,6 +24272,11 @@
         </is>
       </c>
       <c r="EA26" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB26" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -24768,6 +25098,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE27" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF27" t="inlineStr">
         <is>
           <t>O</t>
@@ -24848,6 +25183,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV27" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW27" t="inlineStr">
         <is>
           <t>O</t>
@@ -24869,6 +25209,11 @@
         </is>
       </c>
       <c r="EA27" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB27" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -25690,6 +26035,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE28" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF28" t="inlineStr">
         <is>
           <t>O</t>
@@ -25770,6 +26120,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV28" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW28" t="inlineStr">
         <is>
           <t>O</t>
@@ -25791,6 +26146,11 @@
         </is>
       </c>
       <c r="EA28" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB28" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -26617,6 +26977,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF29" t="inlineStr">
         <is>
           <t>O</t>
@@ -26697,6 +27062,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW29" t="inlineStr">
         <is>
           <t>O</t>
@@ -26718,6 +27088,11 @@
         </is>
       </c>
       <c r="EA29" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB29" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -27544,6 +27919,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE30" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF30" t="inlineStr">
         <is>
           <t>O</t>
@@ -27624,6 +28004,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV30" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW30" t="inlineStr">
         <is>
           <t>O</t>
@@ -27645,6 +28030,11 @@
         </is>
       </c>
       <c r="EA30" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB30" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -28471,6 +28861,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE31" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF31" t="inlineStr">
         <is>
           <t>O</t>
@@ -28551,6 +28946,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV31" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW31" t="inlineStr">
         <is>
           <t>N</t>
@@ -28572,6 +28972,11 @@
         </is>
       </c>
       <c r="EA31" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB31" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -29398,6 +29803,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE32" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF32" t="inlineStr">
         <is>
           <t>O</t>
@@ -29478,6 +29888,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV32" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW32" t="inlineStr">
         <is>
           <t>N</t>
@@ -29499,6 +29914,11 @@
         </is>
       </c>
       <c r="EA32" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB32" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -30325,6 +30745,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE33" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF33" t="inlineStr">
         <is>
           <t>O</t>
@@ -30405,6 +30830,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV33" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW33" t="inlineStr">
         <is>
           <t>N</t>
@@ -30426,6 +30856,11 @@
         </is>
       </c>
       <c r="EA33" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB33" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -31252,6 +31687,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE34" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF34" t="inlineStr">
         <is>
           <t>O</t>
@@ -31332,6 +31772,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV34" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW34" t="inlineStr">
         <is>
           <t>N</t>
@@ -31353,6 +31798,11 @@
         </is>
       </c>
       <c r="EA34" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB34" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -32179,6 +32629,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF35" t="inlineStr">
         <is>
           <t>O</t>
@@ -32259,6 +32714,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW35" t="inlineStr">
         <is>
           <t>N</t>
@@ -32280,6 +32740,11 @@
         </is>
       </c>
       <c r="EA35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB35" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -33106,6 +33571,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE36" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF36" t="inlineStr">
         <is>
           <t>O</t>
@@ -33186,6 +33656,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV36" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW36" t="inlineStr">
         <is>
           <t>N</t>
@@ -33207,6 +33682,11 @@
         </is>
       </c>
       <c r="EA36" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB36" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -34033,6 +34513,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF37" t="inlineStr">
         <is>
           <t>O</t>
@@ -34113,6 +34598,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW37" t="inlineStr">
         <is>
           <t>N</t>
@@ -34134,6 +34624,11 @@
         </is>
       </c>
       <c r="EA37" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB37" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -34960,6 +35455,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF38" t="inlineStr">
         <is>
           <t>O</t>
@@ -35040,6 +35540,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW38" t="inlineStr">
         <is>
           <t>N</t>
@@ -35061,6 +35566,11 @@
         </is>
       </c>
       <c r="EA38" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB38" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -35887,6 +36397,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE39" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF39" t="inlineStr">
         <is>
           <t>O</t>
@@ -35967,6 +36482,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV39" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW39" t="inlineStr">
         <is>
           <t>N</t>
@@ -35988,6 +36508,11 @@
         </is>
       </c>
       <c r="EA39" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB39" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -36814,6 +37339,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF40" t="inlineStr">
         <is>
           <t>O</t>
@@ -36894,6 +37424,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW40" t="inlineStr">
         <is>
           <t>N</t>
@@ -36915,6 +37450,11 @@
         </is>
       </c>
       <c r="EA40" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB40" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -37741,6 +38281,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF41" t="inlineStr">
         <is>
           <t>O</t>
@@ -37821,6 +38366,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW41" t="inlineStr">
         <is>
           <t>N</t>
@@ -37842,6 +38392,11 @@
         </is>
       </c>
       <c r="EA41" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB41" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -38668,6 +39223,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF42" t="inlineStr">
         <is>
           <t>O</t>
@@ -38748,6 +39308,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW42" t="inlineStr">
         <is>
           <t>N</t>
@@ -38769,6 +39334,11 @@
         </is>
       </c>
       <c r="EA42" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB42" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -39595,6 +40165,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE43" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF43" t="inlineStr">
         <is>
           <t>O</t>
@@ -39675,6 +40250,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV43" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW43" t="inlineStr">
         <is>
           <t>N</t>
@@ -39696,6 +40276,11 @@
         </is>
       </c>
       <c r="EA43" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB43" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -40522,6 +41107,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE44" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF44" t="inlineStr">
         <is>
           <t>O</t>
@@ -40602,6 +41192,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV44" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW44" t="inlineStr">
         <is>
           <t>N</t>
@@ -40623,6 +41218,11 @@
         </is>
       </c>
       <c r="EA44" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB44" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -41449,6 +42049,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE45" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF45" t="inlineStr">
         <is>
           <t>O</t>
@@ -41529,6 +42134,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV45" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW45" t="inlineStr">
         <is>
           <t>N</t>
@@ -41550,6 +42160,11 @@
         </is>
       </c>
       <c r="EA45" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB45" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -42376,6 +42991,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE46" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF46" t="inlineStr">
         <is>
           <t>O</t>
@@ -42456,6 +43076,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV46" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW46" t="inlineStr">
         <is>
           <t>N</t>
@@ -42477,6 +43102,11 @@
         </is>
       </c>
       <c r="EA46" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB46" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -43303,6 +43933,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE47" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF47" t="inlineStr">
         <is>
           <t>O</t>
@@ -43383,6 +44018,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV47" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW47" t="inlineStr">
         <is>
           <t>N</t>
@@ -43404,6 +44044,11 @@
         </is>
       </c>
       <c r="EA47" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB47" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -44230,6 +44875,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE48" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF48" t="inlineStr">
         <is>
           <t>O</t>
@@ -44310,6 +44960,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV48" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW48" t="inlineStr">
         <is>
           <t>N</t>
@@ -44331,6 +44986,11 @@
         </is>
       </c>
       <c r="EA48" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB48" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -45157,6 +45817,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF49" t="inlineStr">
         <is>
           <t>O</t>
@@ -45237,6 +45902,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW49" t="inlineStr">
         <is>
           <t>N</t>
@@ -45258,6 +45928,11 @@
         </is>
       </c>
       <c r="EA49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB49" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -46084,6 +46759,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF50" t="inlineStr">
         <is>
           <t>O</t>
@@ -46164,6 +46844,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW50" t="inlineStr">
         <is>
           <t>N</t>
@@ -46185,6 +46870,11 @@
         </is>
       </c>
       <c r="EA50" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB50" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -47011,6 +47701,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF51" t="inlineStr">
         <is>
           <t>O</t>
@@ -47091,6 +47786,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW51" t="inlineStr">
         <is>
           <t>N</t>
@@ -47112,6 +47812,11 @@
         </is>
       </c>
       <c r="EA51" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB51" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -47938,6 +48643,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE52" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF52" t="inlineStr">
         <is>
           <t>O</t>
@@ -48018,6 +48728,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV52" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW52" t="inlineStr">
         <is>
           <t>N</t>
@@ -48039,6 +48754,11 @@
         </is>
       </c>
       <c r="EA52" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB52" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -48865,6 +49585,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF53" t="inlineStr">
         <is>
           <t>O</t>
@@ -48945,6 +49670,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW53" t="inlineStr">
         <is>
           <t>N</t>
@@ -48966,6 +49696,11 @@
         </is>
       </c>
       <c r="EA53" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB53" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -49792,6 +50527,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE54" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF54" t="inlineStr">
         <is>
           <t>O</t>
@@ -49872,6 +50612,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV54" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW54" t="inlineStr">
         <is>
           <t>N</t>
@@ -49893,6 +50638,11 @@
         </is>
       </c>
       <c r="EA54" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB54" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -50719,6 +51469,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF55" t="inlineStr">
         <is>
           <t>O</t>
@@ -50799,6 +51554,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW55" t="inlineStr">
         <is>
           <t>N</t>
@@ -50820,6 +51580,11 @@
         </is>
       </c>
       <c r="EA55" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB55" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -51646,6 +52411,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE56" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF56" t="inlineStr">
         <is>
           <t>O</t>
@@ -51726,6 +52496,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV56" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW56" t="inlineStr">
         <is>
           <t>N</t>
@@ -51747,6 +52522,11 @@
         </is>
       </c>
       <c r="EA56" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB56" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -52573,6 +53353,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE57" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF57" t="inlineStr">
         <is>
           <t>O</t>
@@ -52653,6 +53438,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV57" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW57" t="inlineStr">
         <is>
           <t>N</t>
@@ -52674,6 +53464,11 @@
         </is>
       </c>
       <c r="EA57" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB57" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -53500,6 +54295,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF58" t="inlineStr">
         <is>
           <t>O</t>
@@ -53580,6 +54380,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW58" t="inlineStr">
         <is>
           <t>N</t>
@@ -53601,6 +54406,11 @@
         </is>
       </c>
       <c r="EA58" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB58" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -54427,6 +55237,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE59" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF59" t="inlineStr">
         <is>
           <t>O</t>
@@ -54507,6 +55322,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV59" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW59" t="inlineStr">
         <is>
           <t>N</t>
@@ -54528,6 +55348,11 @@
         </is>
       </c>
       <c r="EA59" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB59" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -55354,6 +56179,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE60" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF60" t="inlineStr">
         <is>
           <t>O</t>
@@ -55434,6 +56264,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV60" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW60" t="inlineStr">
         <is>
           <t>N</t>
@@ -55455,6 +56290,11 @@
         </is>
       </c>
       <c r="EA60" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB60" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -56281,6 +57121,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE61" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF61" t="inlineStr">
         <is>
           <t>O</t>
@@ -56361,6 +57206,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV61" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW61" t="inlineStr">
         <is>
           <t>N</t>
@@ -56382,6 +57232,11 @@
         </is>
       </c>
       <c r="EA61" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB61" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -57208,6 +58063,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE62" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF62" t="inlineStr">
         <is>
           <t>O</t>
@@ -57288,6 +58148,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV62" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW62" t="inlineStr">
         <is>
           <t>N</t>
@@ -57309,6 +58174,11 @@
         </is>
       </c>
       <c r="EA62" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB62" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -58135,6 +59005,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE63" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF63" t="inlineStr">
         <is>
           <t>O</t>
@@ -58215,6 +59090,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV63" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW63" t="inlineStr">
         <is>
           <t>N</t>
@@ -58236,6 +59116,11 @@
         </is>
       </c>
       <c r="EA63" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB63" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -59062,6 +59947,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF64" t="inlineStr">
         <is>
           <t>O</t>
@@ -59142,6 +60032,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW64" t="inlineStr">
         <is>
           <t>N</t>
@@ -59163,6 +60058,11 @@
         </is>
       </c>
       <c r="EA64" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB64" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -59989,6 +60889,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE65" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF65" t="inlineStr">
         <is>
           <t>O</t>
@@ -60069,6 +60974,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV65" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW65" t="inlineStr">
         <is>
           <t>N</t>
@@ -60090,6 +61000,11 @@
         </is>
       </c>
       <c r="EA65" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB65" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -60916,6 +61831,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE66" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF66" t="inlineStr">
         <is>
           <t>O</t>
@@ -60996,6 +61916,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV66" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW66" t="inlineStr">
         <is>
           <t>N</t>
@@ -61017,6 +61942,11 @@
         </is>
       </c>
       <c r="EA66" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB66" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -61843,6 +62773,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE67" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF67" t="inlineStr">
         <is>
           <t>O</t>
@@ -61923,6 +62858,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV67" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW67" t="inlineStr">
         <is>
           <t>N</t>
@@ -61944,6 +62884,11 @@
         </is>
       </c>
       <c r="EA67" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB67" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -62770,6 +63715,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE68" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF68" t="inlineStr">
         <is>
           <t>O</t>
@@ -62850,6 +63800,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV68" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW68" t="inlineStr">
         <is>
           <t>N</t>
@@ -62871,6 +63826,11 @@
         </is>
       </c>
       <c r="EA68" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB68" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -63697,6 +64657,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE69" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF69" t="inlineStr">
         <is>
           <t>O</t>
@@ -63777,6 +64742,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV69" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW69" t="inlineStr">
         <is>
           <t>N</t>
@@ -63798,6 +64768,11 @@
         </is>
       </c>
       <c r="EA69" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB69" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -64624,6 +65599,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE70" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF70" t="inlineStr">
         <is>
           <t>O</t>
@@ -64704,6 +65684,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV70" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW70" t="inlineStr">
         <is>
           <t>N</t>
@@ -64725,6 +65710,11 @@
         </is>
       </c>
       <c r="EA70" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB70" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -65551,6 +66541,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE71" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF71" t="inlineStr">
         <is>
           <t>O</t>
@@ -65631,6 +66626,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV71" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW71" t="inlineStr">
         <is>
           <t>N</t>
@@ -65652,6 +66652,11 @@
         </is>
       </c>
       <c r="EA71" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB71" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -66478,6 +67483,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE72" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF72" t="inlineStr">
         <is>
           <t>O</t>
@@ -66558,6 +67568,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV72" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW72" t="inlineStr">
         <is>
           <t>N</t>
@@ -66579,6 +67594,11 @@
         </is>
       </c>
       <c r="EA72" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB72" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -67405,6 +68425,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE73" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF73" t="inlineStr">
         <is>
           <t>O</t>
@@ -67485,6 +68510,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV73" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW73" t="inlineStr">
         <is>
           <t>N</t>
@@ -67506,6 +68536,11 @@
         </is>
       </c>
       <c r="EA73" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB73" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -68332,6 +69367,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE74" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF74" t="inlineStr">
         <is>
           <t>O</t>
@@ -68412,6 +69452,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV74" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW74" t="inlineStr">
         <is>
           <t>N</t>
@@ -68433,6 +69478,11 @@
         </is>
       </c>
       <c r="EA74" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB74" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -69259,6 +70309,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE75" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF75" t="inlineStr">
         <is>
           <t>O</t>
@@ -69339,6 +70394,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV75" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW75" t="inlineStr">
         <is>
           <t>N</t>
@@ -69360,6 +70420,11 @@
         </is>
       </c>
       <c r="EA75" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB75" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -70186,6 +71251,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE76" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF76" t="inlineStr">
         <is>
           <t>O</t>
@@ -70266,6 +71336,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV76" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW76" t="inlineStr">
         <is>
           <t>N</t>
@@ -70287,6 +71362,11 @@
         </is>
       </c>
       <c r="EA76" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB76" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -71113,6 +72193,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE77" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF77" t="inlineStr">
         <is>
           <t>O</t>
@@ -71193,6 +72278,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV77" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW77" t="inlineStr">
         <is>
           <t>N</t>
@@ -71214,6 +72304,11 @@
         </is>
       </c>
       <c r="EA77" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB77" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -72040,6 +73135,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE78" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF78" t="inlineStr">
         <is>
           <t>O</t>
@@ -72120,6 +73220,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV78" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW78" t="inlineStr">
         <is>
           <t>N</t>
@@ -72141,6 +73246,11 @@
         </is>
       </c>
       <c r="EA78" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB78" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -72967,6 +74077,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE79" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF79" t="inlineStr">
         <is>
           <t>O</t>
@@ -73047,6 +74162,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV79" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW79" t="inlineStr">
         <is>
           <t>N</t>
@@ -73068,6 +74188,11 @@
         </is>
       </c>
       <c r="EA79" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB79" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -73894,6 +75019,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE80" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF80" t="inlineStr">
         <is>
           <t>O</t>
@@ -73974,6 +75104,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV80" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW80" t="inlineStr">
         <is>
           <t>N</t>
@@ -73995,6 +75130,11 @@
         </is>
       </c>
       <c r="EA80" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB80" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -74821,6 +75961,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE81" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF81" t="inlineStr">
         <is>
           <t>O</t>
@@ -74901,6 +76046,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV81" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW81" t="inlineStr">
         <is>
           <t>N</t>
@@ -74922,6 +76072,11 @@
         </is>
       </c>
       <c r="EA81" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB81" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -75748,6 +76903,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE82" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF82" t="inlineStr">
         <is>
           <t>O</t>
@@ -75828,6 +76988,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV82" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW82" t="inlineStr">
         <is>
           <t>N</t>
@@ -75849,6 +77014,11 @@
         </is>
       </c>
       <c r="EA82" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB82" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -76675,6 +77845,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE83" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF83" t="inlineStr">
         <is>
           <t>O</t>
@@ -76755,6 +77930,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV83" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW83" t="inlineStr">
         <is>
           <t>N</t>
@@ -76776,6 +77956,11 @@
         </is>
       </c>
       <c r="EA83" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB83" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -77602,6 +78787,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE84" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF84" t="inlineStr">
         <is>
           <t>O</t>
@@ -77682,6 +78872,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV84" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW84" t="inlineStr">
         <is>
           <t>N</t>
@@ -77703,6 +78898,11 @@
         </is>
       </c>
       <c r="EA84" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB84" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -78529,6 +79729,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE85" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF85" t="inlineStr">
         <is>
           <t>O</t>
@@ -78609,6 +79814,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV85" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW85" t="inlineStr">
         <is>
           <t>N</t>
@@ -78630,6 +79840,11 @@
         </is>
       </c>
       <c r="EA85" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB85" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -79456,6 +80671,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE86" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF86" t="inlineStr">
         <is>
           <t>O</t>
@@ -79536,6 +80756,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV86" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW86" t="inlineStr">
         <is>
           <t>N</t>
@@ -79557,6 +80782,11 @@
         </is>
       </c>
       <c r="EA86" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB86" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -80383,6 +81613,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE87" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF87" t="inlineStr">
         <is>
           <t>O</t>
@@ -80463,6 +81698,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV87" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW87" t="inlineStr">
         <is>
           <t>N</t>
@@ -80484,6 +81724,11 @@
         </is>
       </c>
       <c r="EA87" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB87" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -81310,6 +82555,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE88" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF88" t="inlineStr">
         <is>
           <t>O</t>
@@ -81390,6 +82640,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV88" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW88" t="inlineStr">
         <is>
           <t>N</t>
@@ -81411,6 +82666,11 @@
         </is>
       </c>
       <c r="EA88" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB88" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -82237,6 +83497,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE89" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF89" t="inlineStr">
         <is>
           <t>O</t>
@@ -82317,6 +83582,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV89" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW89" t="inlineStr">
         <is>
           <t>N</t>
@@ -82338,6 +83608,11 @@
         </is>
       </c>
       <c r="EA89" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB89" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -83164,6 +84439,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE90" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF90" t="inlineStr">
         <is>
           <t>O</t>
@@ -83244,6 +84524,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV90" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW90" t="inlineStr">
         <is>
           <t>N</t>
@@ -83265,6 +84550,11 @@
         </is>
       </c>
       <c r="EA90" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB90" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -84091,6 +85381,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DE91" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DF91" t="inlineStr">
         <is>
           <t>O</t>
@@ -84171,6 +85466,11 @@
           <t>N</t>
         </is>
       </c>
+      <c r="DV91" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
       <c r="DW91" t="inlineStr">
         <is>
           <t>N</t>
@@ -84192,6 +85492,11 @@
         </is>
       </c>
       <c r="EA91" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="EB91" t="inlineStr">
         <is>
           <t>N</t>
         </is>

</xml_diff>